<commit_message>
feat: add example rows to Excel import template
Show all action types (buy, sell, dividend with withholding tax, fee)
with amber styling and a note to delete before importing.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -35,13 +35,64 @@
   </si>
   <si>
     <t>Currency</t>
+  </si>
+  <si>
+    <t>2025-01-10</t>
+  </si>
+  <si>
+    <t>AAPL</t>
+  </si>
+  <si>
+    <t>buy</t>
+  </si>
+  <si>
+    <t>Interactive Brokers</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>2025-02-03</t>
+  </si>
+  <si>
+    <t>MSFT</t>
+  </si>
+  <si>
+    <t>2025-03-15</t>
+  </si>
+  <si>
+    <t>dividend</t>
+  </si>
+  <si>
+    <t>2025-04-01</t>
+  </si>
+  <si>
+    <t>sell</t>
+  </si>
+  <si>
+    <t>2025-04-15</t>
+  </si>
+  <si>
+    <t>VOO</t>
+  </si>
+  <si>
+    <t>Fidelity</t>
+  </si>
+  <si>
+    <t>2025-05-01</t>
+  </si>
+  <si>
+    <t>fee</t>
+  </si>
+  <si>
+    <t>↑ Delete these example rows before importing. Enter your data below.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -52,8 +103,16 @@
     <font>
       <b/>
     </font>
+    <font>
+      <i/>
+      <color rgb="FF92400E"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFDC2626"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -63,6 +122,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4F4F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFBEB"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,9 +142,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,14 +523,200 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="3:3" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2">
+        <v>3450</v>
+      </c>
+      <c r="F2" s="2">
+        <v>4.95</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2">
+        <v>3200</v>
+      </c>
+      <c r="F3" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-0.56</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1200</v>
+      </c>
+      <c r="F6" s="2">
+        <v>4.95</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1500</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>12</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
     <row r="10" spans="3:3" x14ac:dyDescent="0.25"/>
     <row r="11" spans="3:3" x14ac:dyDescent="0.25"/>
     <row r="12" spans="3:3" x14ac:dyDescent="0.25"/>
@@ -1457,6 +1709,9 @@
     <row r="999" spans="3:3" x14ac:dyDescent="0.25"/>
     <row r="1000" spans="3:3" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A9:H9"/>
+  </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" showErrorMessage="1" errorTitle="Invalid Action" error="Must be buy, sell, dividend, or fee" sqref="C10:C1000">
       <formula1>"buy,sell,dividend,fee"</formula1>

</xml_diff>